<commit_message>
Accept a sheet back from Google, and stop it eating unknown fields
Import now takes content/roster.csv as well as roster.xlsx, whichever
was saved last, because Download as CSV is the one-click Google Sheets
export and has nothing to go wrong. The xlsx reader already resolved
shared strings and boolean cells, which is what Sheets and Excel write
where this exporter writes inline strings; that is now verified against
a file built the way they build one.

More importantly, a field the sheet has no column for is carried through
from the current JSON rather than dropped. endsRunChance was added to
the game while this script existed without a column for it, so the next
import would have silently deleted it - which is the one failure a
content pipeline must not have. It has a column now, and anything added
next survives regardless.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HDrKcag3n2pSU2TvDz2jdx
</commit_message>
<xml_diff>
--- a/content/roster.xlsx
+++ b/content/roster.xlsx
@@ -54,7 +54,8 @@
     <col min="10" max="10" width="30" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
     <col min="12" max="12" width="34" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="13" max="13" width="26" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -120,6 +121,11 @@
       </c>
       <c r="M1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">endsRunChance (0-1, blank = certain)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">reviewed (TRUE/FALSE)</t>
         </is>
       </c>
@@ -180,7 +186,7 @@
           <t xml:space="preserve">leopold-ii</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -237,7 +243,7 @@
           <t xml:space="preserve">beloved, statesman, loyalist</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -299,7 +305,7 @@
           <t xml:space="preserve">chamberlain</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -361,7 +367,7 @@
           <t xml:space="preserve">pinochet</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -423,7 +429,7 @@
           <t xml:space="preserve">vlad</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -480,7 +486,7 @@
           <t xml:space="preserve">statesman, soldier, strategist</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -537,7 +543,7 @@
           <t xml:space="preserve">statesman, technocrat, loyalist</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -594,7 +600,7 @@
           <t xml:space="preserve">statesman, beloved, strategist</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -651,7 +657,7 @@
           <t xml:space="preserve">statesman, cunning, showman</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -708,7 +714,7 @@
           <t xml:space="preserve">beloved, showman, statesman</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -765,7 +771,7 @@
           <t xml:space="preserve">beloved, statesman, dealmaker</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -822,7 +828,7 @@
           <t xml:space="preserve">technocrat, statesman, strategist</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -879,7 +885,7 @@
           <t xml:space="preserve">technocrat, statesman, loyalist</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -941,7 +947,7 @@
           <t xml:space="preserve">pinochet</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -998,7 +1004,7 @@
           <t xml:space="preserve">beloved, statesman, showman</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1055,7 +1061,7 @@
           <t xml:space="preserve">statesman, warhawk, strategist</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1112,7 +1118,7 @@
           <t xml:space="preserve">soldier, showman, statesman</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1169,7 +1175,7 @@
           <t xml:space="preserve">soldier, strategist, statesman</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1226,7 +1232,7 @@
           <t xml:space="preserve">dealmaker, statesman, beloved</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1283,7 +1289,7 @@
           <t xml:space="preserve">beloved, statesman, soldier</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1345,7 +1351,7 @@
           <t xml:space="preserve">Eighteen and a half minutes of the tape are missing. So is your government.</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1402,7 +1408,7 @@
           <t xml:space="preserve">warhawk, soldier, strategist</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1464,7 +1470,7 @@
           <t xml:space="preserve">robespierre</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1521,7 +1527,7 @@
           <t xml:space="preserve">demagogue, strategist, paranoid</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1578,7 +1584,7 @@
           <t xml:space="preserve">paranoid, demagogue, isolationist</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1635,7 +1641,7 @@
           <t xml:space="preserve">demagogue, showman, warhawk</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1692,7 +1698,7 @@
           <t xml:space="preserve">paranoid, soldier, isolationist</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1749,7 +1755,7 @@
           <t xml:space="preserve">showman, warhawk, paranoid</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1806,7 +1812,7 @@
           <t xml:space="preserve">paranoid, demagogue, showman</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1868,7 +1874,7 @@
           <t xml:space="preserve">allende, mandela</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1925,7 +1931,7 @@
           <t xml:space="preserve">demagogue, paranoid, showman</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -1982,7 +1988,7 @@
           <t xml:space="preserve">paranoid, demagogue, cunning</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2039,7 +2045,7 @@
           <t xml:space="preserve">showman, demagogue, paranoid</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2096,7 +2102,7 @@
           <t xml:space="preserve">paranoid, warhawk, demagogue</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2153,7 +2159,7 @@
           <t xml:space="preserve">showman, warhawk, paranoid</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2210,7 +2216,7 @@
           <t xml:space="preserve">cunning, showman, dealmaker</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2267,7 +2273,7 @@
           <t xml:space="preserve">cunning, demagogue, banker</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2324,7 +2330,7 @@
           <t xml:space="preserve">showman, demagogue, paranoid</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2386,7 +2392,7 @@
           <t xml:space="preserve">lincoln</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2443,7 +2449,7 @@
           <t xml:space="preserve">showman, paranoid, demagogue</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2505,7 +2511,7 @@
           <t xml:space="preserve">gandhi</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2567,7 +2573,7 @@
           <t xml:space="preserve">stalin</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2629,7 +2635,7 @@
           <t xml:space="preserve">churchill</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2686,7 +2692,7 @@
           <t xml:space="preserve">strategist, cunning, statesman</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2748,7 +2754,7 @@
           <t xml:space="preserve">crassus</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="N46" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2805,7 +2811,7 @@
           <t xml:space="preserve">dealmaker, showman, cunning</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="N47" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2862,7 +2868,7 @@
           <t xml:space="preserve">technocrat, banker, scandal-magnet</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="N48" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2919,7 +2925,7 @@
           <t xml:space="preserve">demagogue, showman, scandal-magnet</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="N49" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -2981,7 +2987,7 @@
           <t xml:space="preserve">caesar</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="N50" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3038,7 +3044,7 @@
           <t xml:space="preserve">dealmaker, cunning, loyalist</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="N51" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3095,7 +3101,7 @@
           <t xml:space="preserve">showman, soldier, paranoid</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="N52" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3152,7 +3158,7 @@
           <t xml:space="preserve">showman, beloved, loyalist</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="N53" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3209,7 +3215,7 @@
           <t xml:space="preserve">banker, dealmaker, showman</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="N54" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3266,7 +3272,7 @@
           <t xml:space="preserve">warhawk, soldier, showman</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="N55" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3323,7 +3329,7 @@
           <t xml:space="preserve">beloved, statesman, loyalist</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="N56" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3380,7 +3386,7 @@
           <t xml:space="preserve">warhawk, soldier, paranoid, strategist</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="N57" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3437,7 +3443,7 @@
           <t xml:space="preserve">beloved, loyalist, statesman</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="N58" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3494,7 +3500,7 @@
           <t xml:space="preserve">dealmaker, beloved, loyalist</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="N59" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3551,7 +3557,7 @@
           <t xml:space="preserve">isolationist, soldier, beloved</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr">
+      <c r="N60" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3613,7 +3619,7 @@
           <t xml:space="preserve">sauron</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
+      <c r="N61" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3675,7 +3681,7 @@
           <t xml:space="preserve">gandalf, optimus-prime</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="N62" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3732,7 +3738,7 @@
           <t xml:space="preserve">statesman, strategist, loyalist</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="N63" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3794,7 +3800,7 @@
           <t xml:space="preserve">joker</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr">
+      <c r="N64" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3856,7 +3862,7 @@
           <t xml:space="preserve">batman</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr">
+      <c r="N65" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3918,7 +3924,7 @@
           <t xml:space="preserve">mr-burns</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr">
+      <c r="N66" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -3980,7 +3986,7 @@
           <t xml:space="preserve">homer-simpson</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
+      <c r="N67" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4037,7 +4043,7 @@
           <t xml:space="preserve">beloved, loyalist, showman</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
+      <c r="N68" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4094,7 +4100,7 @@
           <t xml:space="preserve">liability, beloved, loyalist</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr">
+      <c r="N69" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4156,7 +4162,7 @@
           <t xml:space="preserve">mario</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr">
+      <c r="N70" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4218,7 +4224,7 @@
           <t xml:space="preserve">bowser</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr">
+      <c r="N71" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4275,7 +4281,7 @@
           <t xml:space="preserve">warhawk, soldier, isolationist</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr">
+      <c r="N72" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4337,7 +4343,7 @@
           <t xml:space="preserve">sauron</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr">
+      <c r="N73" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4394,7 +4400,7 @@
           <t xml:space="preserve">warhawk, technocrat, strategist</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr">
+      <c r="N74" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4451,7 +4457,7 @@
           <t xml:space="preserve">technocrat, paranoid, cunning</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr">
+      <c r="N75" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4508,7 +4514,7 @@
           <t xml:space="preserve">technocrat, cunning, demagogue</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr">
+      <c r="N76" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4565,7 +4571,7 @@
           <t xml:space="preserve">strategist, technocrat, paranoid</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr">
+      <c r="N77" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4622,7 +4628,7 @@
           <t xml:space="preserve">cunning, showman, isolationist</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr">
+      <c r="N78" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4679,7 +4685,7 @@
           <t xml:space="preserve">beloved, loyalist, liability</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr">
+      <c r="N79" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4736,7 +4742,7 @@
           <t xml:space="preserve">paranoid, cunning, liability</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr">
+      <c r="N80" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4793,7 +4799,7 @@
           <t xml:space="preserve">paranoid, demagogue, warhawk</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr">
+      <c r="N81" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4850,7 +4856,7 @@
           <t xml:space="preserve">cunning, technocrat, paranoid</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr">
+      <c r="N82" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4907,7 +4913,7 @@
           <t xml:space="preserve">isolationist, warhawk, paranoid</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr">
+      <c r="N83" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -4964,7 +4970,7 @@
           <t xml:space="preserve">liability, loyalist, beloved</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr">
+      <c r="N84" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5021,7 +5027,7 @@
           <t xml:space="preserve">soldier, showman, beloved</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr">
+      <c r="N85" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5078,7 +5084,7 @@
           <t xml:space="preserve">paranoid, loyalist, liability</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr">
+      <c r="N86" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5135,7 +5141,7 @@
           <t xml:space="preserve">technocrat, soldier, loyalist</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr">
+      <c r="N87" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5192,7 +5198,7 @@
           <t xml:space="preserve">showman, technocrat, scandal-magnet</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr">
+      <c r="N88" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5249,7 +5255,7 @@
           <t xml:space="preserve">showman, dealmaker, beloved</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr">
+      <c r="N89" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5306,7 +5312,7 @@
           <t xml:space="preserve">beloved, showman, soldier</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr">
+      <c r="N90" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5363,7 +5369,7 @@
           <t xml:space="preserve">beloved, dealmaker, showman</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr">
+      <c r="N91" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5420,7 +5426,7 @@
           <t xml:space="preserve">beloved, statesman, technocrat</t>
         </is>
       </c>
-      <c r="M92" t="inlineStr">
+      <c r="N92" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5477,7 +5483,7 @@
           <t xml:space="preserve">beloved, soldier, showman</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr">
+      <c r="N93" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5534,7 +5540,7 @@
           <t xml:space="preserve">beloved, statesman, loyalist</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr">
+      <c r="N94" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5591,7 +5597,7 @@
           <t xml:space="preserve">technocrat, showman, soldier</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr">
+      <c r="N95" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5648,7 +5654,7 @@
           <t xml:space="preserve">technocrat, paranoid, strategist</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr">
+      <c r="N96" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5705,7 +5711,7 @@
           <t xml:space="preserve">technocrat, statesman, beloved</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr">
+      <c r="N97" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5762,7 +5768,7 @@
           <t xml:space="preserve">technocrat, strategist, banker</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr">
+      <c r="N98" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5819,7 +5825,7 @@
           <t xml:space="preserve">technocrat, loyalist, statesman</t>
         </is>
       </c>
-      <c r="M99" t="inlineStr">
+      <c r="N99" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5876,7 +5882,7 @@
           <t xml:space="preserve">technocrat, strategist, loyalist</t>
         </is>
       </c>
-      <c r="M100" t="inlineStr">
+      <c r="N100" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5933,7 +5939,7 @@
           <t xml:space="preserve">statesman, beloved, technocrat</t>
         </is>
       </c>
-      <c r="M101" t="inlineStr">
+      <c r="N101" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -5990,7 +5996,7 @@
           <t xml:space="preserve">showman, dealmaker, beloved</t>
         </is>
       </c>
-      <c r="M102" t="inlineStr">
+      <c r="N102" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6047,7 +6053,7 @@
           <t xml:space="preserve">showman, soldier, liability</t>
         </is>
       </c>
-      <c r="M103" t="inlineStr">
+      <c r="N103" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6104,7 +6110,7 @@
           <t xml:space="preserve">statesman, strategist, isolationist</t>
         </is>
       </c>
-      <c r="M104" t="inlineStr">
+      <c r="N104" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6161,7 +6167,7 @@
           <t xml:space="preserve">showman, beloved, demagogue</t>
         </is>
       </c>
-      <c r="M105" t="inlineStr">
+      <c r="N105" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6218,7 +6224,7 @@
           <t xml:space="preserve">soldier, showman, strategist</t>
         </is>
       </c>
-      <c r="M106" t="inlineStr">
+      <c r="N106" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6275,7 +6281,7 @@
           <t xml:space="preserve">demagogue, showman, scandal-magnet</t>
         </is>
       </c>
-      <c r="M107" t="inlineStr">
+      <c r="N107" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6332,7 +6338,7 @@
           <t xml:space="preserve">statesman, soldier, technocrat</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr">
+      <c r="N108" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6389,7 +6395,7 @@
           <t xml:space="preserve">demagogue, cunning, showman</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr">
+      <c r="N109" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6446,7 +6452,7 @@
           <t xml:space="preserve">showman, dealmaker, banker</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr">
+      <c r="N110" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6503,7 +6509,7 @@
           <t xml:space="preserve">showman, demagogue, soldier</t>
         </is>
       </c>
-      <c r="M111" t="inlineStr">
+      <c r="N111" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6560,7 +6566,7 @@
           <t xml:space="preserve">dealmaker, banker, loyalist</t>
         </is>
       </c>
-      <c r="M112" t="inlineStr">
+      <c r="N112" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6617,7 +6623,7 @@
           <t xml:space="preserve">statesman, strategist, paranoid</t>
         </is>
       </c>
-      <c r="M113" t="inlineStr">
+      <c r="N113" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6674,7 +6680,7 @@
           <t xml:space="preserve">loyalist, technocrat, liability</t>
         </is>
       </c>
-      <c r="M114" t="inlineStr">
+      <c r="N114" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6731,7 +6737,7 @@
           <t xml:space="preserve">paranoid, technocrat, banker</t>
         </is>
       </c>
-      <c r="M115" t="inlineStr">
+      <c r="N115" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6788,7 +6794,7 @@
           <t xml:space="preserve">loyalist, liability, soldier</t>
         </is>
       </c>
-      <c r="M116" t="inlineStr">
+      <c r="N116" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6845,7 +6851,7 @@
           <t xml:space="preserve">technocrat, loyalist, liability</t>
         </is>
       </c>
-      <c r="M117" t="inlineStr">
+      <c r="N117" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6902,7 +6908,7 @@
           <t xml:space="preserve">technocrat, isolationist, liability</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr">
+      <c r="N118" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -6959,7 +6965,7 @@
           <t xml:space="preserve">loyalist, paranoid, liability</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr">
+      <c r="N119" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -7016,7 +7022,7 @@
           <t xml:space="preserve">cunning, loyalist, scandal-magnet</t>
         </is>
       </c>
-      <c r="M120" t="inlineStr">
+      <c r="N120" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -7073,7 +7079,7 @@
           <t xml:space="preserve">banker, dealmaker, scandal-magnet</t>
         </is>
       </c>
-      <c r="M121" t="inlineStr">
+      <c r="N121" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -7130,7 +7136,7 @@
           <t xml:space="preserve">warhawk, soldier, paranoid</t>
         </is>
       </c>
-      <c r="M122" t="inlineStr">
+      <c r="N122" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
@@ -7187,14 +7193,14 @@
           <t xml:space="preserve">liability, loyalist, beloved</t>
         </is>
       </c>
-      <c r="M123" t="inlineStr">
+      <c r="N123" t="inlineStr">
         <is>
           <t xml:space="preserve">TRUE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M123"/>
+  <autoFilter ref="A1:N123"/>
 </worksheet>
 </file>
 

</xml_diff>